<commit_message>
Reprocess refreshed ruby xlsx bundle
Agent-Logs-Url: https://github.com/Linden10/misc_game-chs/sessions/b24273f5-2c2c-4bfd-8da8-0525a2cfb0c5

Co-authored-by: Linden10 <20895359+Linden10@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/processed_ruby_restored_xlsx/sc000_学級日誌.ss.xlsx
+++ b/processed_ruby_restored_xlsx/sc000_学級日誌.ss.xlsx
@@ -967,7 +967,7 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>sc201_Shared1 - Morning of the Fireworks Festival</t>
+          <t>sc201_Shared1： Morning of the Fireworks Festival</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>sc202_Shared2 - Before the Stargazing Route Split</t>
+          <t>sc202_Shared2： Stargazing Route Before Branch</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1147,8 +1147,8 @@
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>sc203_Shared3 - Before the Amusement Park Route Split
-with Everyone</t>
+          <t>sc203_Shared3： Everyone to the Amusement Park Route
+Before Branch</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
-          <t>sc201_Shared1 - Morning of the Fireworks Festival</t>
+          <t>sc201_Shared1： The morning of the fireworks festival</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -1418,7 +1418,8 @@
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>sc202_Shared2 - Before the Stargazing Route Split</t>
+          <t>sc202_Shared2： Before Astronomical Observation Route
+Split</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -1463,8 +1464,8 @@
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>sc203_Shared3 - Before the Amusement Park Route Split
-with Everyone</t>
+          <t>sc203_shared3： before the amusement-park route split
+with everyone</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -1749,7 +1750,7 @@
       </c>
       <c r="B86" s="1" t="inlineStr">
         <is>
-          <t>sc201_Shared1 - Morning of the Fireworks Festival</t>
+          <t>sc201_Shared1： Morning of the Fireworks Festival</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -1794,7 +1795,7 @@
       </c>
       <c r="B89" s="1" t="inlineStr">
         <is>
-          <t>sc202_Shared2 - Before the Stargazing Route Split</t>
+          <t>sc202_Shared2： Stargazing Route Before Branch</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -1899,8 +1900,8 @@
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>sc203_Shared3 - Before the Amusement Park Route Split
-with Everyone</t>
+          <t>sc203_Shared 3： Before the Amusement Park Route
+Branch with Everyone</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -2095,7 +2096,7 @@
       </c>
       <c r="B109" s="1" t="inlineStr">
         <is>
-          <t>sc201_Shared1 - Morning of the Fireworks Festival</t>
+          <t>sc201_Shared1： Morning of the fireworks festival</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -2140,7 +2141,7 @@
       </c>
       <c r="B112" s="1" t="inlineStr">
         <is>
-          <t>sc202_Shared2 - Before the Stargazing Route Split</t>
+          <t>sc202_Shared2： Stargazing - before route split</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -2275,8 +2276,8 @@
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>sc203_Shared3 - Before the Amusement Park Route Split
-with Everyone</t>
+          <t>sc203_Shared3： Amusement park with everyone - before
+route split</t>
         </is>
       </c>
       <c r="C121" t="n">

</xml_diff>